<commit_message>
fix(client-detail): family SKU breakdown uses gmv.orders + normalised productCode
</commit_message>
<xml_diff>
--- a/Paliers and gifts.xlsx
+++ b/Paliers and gifts.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://beyondbelievers-my.sharepoint.com/personal/k_saguem_z_systems/Documents/Bureau/Rehab app ( planner) - Copie/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{7592EA91-3E94-48F8-8C06-4F4519890483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{341A06E6-6275-44C9-A32E-60FE5C46FE2E}"/>
+  <xr:revisionPtr revIDLastSave="3" documentId="8_{7592EA91-3E94-48F8-8C06-4F4519890483}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8A9D34A-D762-4A25-8D85-8FC7F60C2019}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{C67AB8F8-37BF-4CA2-862C-01203FF86119}"/>
   </bookViews>
@@ -52,6 +52,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/karcher-nettoyeur-haute-pression-k2-edition-universelle-canon-a-mousse-brosse-de-nettoyage-des-jantes-offerts-67806363.html</t>
         </r>
@@ -65,6 +66,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/karcher-nettoyeur-haute-pression-k2-edition-universelle-canon-a-mousse-brosse-de-nettoyage-des-jantes-offerts-67806363.html</t>
         </r>
@@ -78,6 +80,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/rowenta-aspirateur-robot-laveur-x-plorer-serie85-rr87c5wh-67826912.html</t>
         </r>
@@ -91,6 +94,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/karcher-nettoyeur-haute-pression-k2-edition-universelle-canon-a-mousse-brosse-de-nettoyage-des-jantes-offerts-67806363.html</t>
         </r>
@@ -104,6 +108,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/rowenta-aspirateur-robot-laveur-x-plorer-serie85-rr87c5wh-67826912.html</t>
         </r>
@@ -117,6 +122,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/delonghi-magnifica-start-machine-espresso-full-automatique-avec-bro-67248497.html</t>
         </r>
@@ -130,6 +136,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/sharp-machine-a-laver-7kg-1200-trmin-67172734.html</t>
         </r>
@@ -143,6 +150,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/thomson-google-tv-55-qled-pro-67246900.html</t>
         </r>
@@ -156,6 +164,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/infiniton-refrigerateur-americain-sbs-668-wdix-no-frost-177-cm-559-l-64693450.html</t>
         </r>
@@ -169,6 +178,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/rowenta-aspirateur-robot-laveur-x-plorer-serie85-rr87c5wh-67826912.html</t>
         </r>
@@ -182,6 +192,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/delonghi-magnifica-start-machine-espresso-full-automatique-avec-bro-67248497.html</t>
         </r>
@@ -195,6 +206,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/85-crystal-uhd-4k-smart-tv-one-ui-tizen-hdr10-design-metalstream-support-gratuit-85u8075-samsung-mpg1544628.html
 https://www.jumia.ma/prima-hotte-60-cm-65430885.html</t>
@@ -209,6 +221,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/hisense-smart-tv-qled-4k-55-garantie-24-mois-67313922.html</t>
         </r>
@@ -222,6 +235,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/75-crystal-uhd-4k-smart-tv-one-ui-tizen-hdr10-design-metalstream-support-gratuit-75u8075-samsung-mpg1544568.html</t>
         </r>
@@ -235,6 +249,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/infiniton-refrigerateur-americain-sbs-668-wdix-no-frost-177-cm-559-l-64693450.html</t>
         </r>
@@ -248,6 +263,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/thomson-google-tv-55-qled-pro-67246900.html</t>
         </r>
@@ -261,6 +277,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/infiniton-refrigerateur-americain-sbs-668-wdix-no-frost-177-cm-559-l-64693450.html</t>
         </r>
@@ -274,6 +291,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/rowenta-aspirateur-robot-laveur-x-plorer-serie85-rr87c5wh-67826912.html</t>
         </r>
@@ -287,6 +305,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/krups-expresso-avec-broyeur-evidence-ea890810-57273607.html</t>
         </r>
@@ -300,6 +319,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-tab-s10-ultra-14.6-12-go-512-go-gris-pierre-de-lune-67308129.html
 https://www.jumia.ma/prima-blender-16l-rouge-60827922.html</t>
@@ -314,6 +334,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/delonghi-magnifica-start-machine-espresso-full-automatique-avec-bro-67248497.html</t>
         </r>
@@ -327,6 +348,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-75-4k-uhd-crystal-smart-tv-tizen-hdr10-son-ots-lite-design-metalstream-support-gratuit-75u8000f-67407815.html
 https://www.jumia.ma/casio-montre-hommes-mtp-v004d-1b2udf-37030865.html</t>
@@ -341,6 +363,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-s26-ultra-69-16gb-ram-1-tb-rom-cobalt-violet-67758540.html</t>
         </r>
@@ -354,6 +377,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/85-crystal-uhd-4k-smart-tv-one-ui-tizen-hdr10-design-metalstream-support-gratuit-85u8075-samsung-mpg1544628.html
 https://www.jumia.ma/prima-hotte-60-cm-65430885.html</t>
@@ -368,6 +392,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/75-crystal-uhd-4k-smart-tv-one-ui-tizen-hdr10-design-metalstream-support-gratuit-75u8075-samsung-mpg1544568.html</t>
         </r>
@@ -381,6 +406,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>Kamal SAGUEM:</t>
         </r>
@@ -389,6 +415,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html</t>
@@ -403,6 +430,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html</t>
         </r>
@@ -416,6 +444,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/infiniton-refrigerateur-americain-sbs-668-wdix-no-frost-177-cm-559-l-64693450.html</t>
         </r>
@@ -429,6 +458,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/rowenta-aspirateur-robot-laveur-x-plorer-serie85-rr87c5wh-67826912.html</t>
         </r>
@@ -442,6 +472,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html
 https://www.jumia.ma/samsung-75-4k-uhd-crystal-smart-tv-tizen-hdr10-son-ots-lite-design-metalstream-support-gratuit-75u8000f-67407815.html
@@ -457,6 +488,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-tab-s10-ultra-14.6-12-go-256-go-gris-pierre-de-lune-67308128.html</t>
         </r>
@@ -470,6 +502,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/thomson-google-tv-55-qled-pro-67246900.html</t>
         </r>
@@ -483,6 +516,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html
 https://www.jumia.ma/samsung-tab-s10-ultra-14.6-12-go-256-go-gris-pierre-de-lune-67308128.html</t>
@@ -497,6 +531,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/85-crystal-uhd-4k-smart-tv-one-ui-tizen-hdr10-design-metalstream-support-gratuit-85u8075-samsung-mpg1544628.html
 https://www.jumia.ma/prima-hotte-60-cm-65430885.html</t>
@@ -511,6 +546,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/infiniton-refrigerateur-americain-sbs-668-wdix-no-frost-177-cm-559-l-64693450.html</t>
         </r>
@@ -524,6 +560,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html
 https://www.jumia.ma/samsung-galaxy-s26-ultra-69-16gb-ram-1-tb-rom-cobalt-violet-67758540.html
@@ -539,6 +576,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>Kamal SAGUEM:</t>
         </r>
@@ -547,6 +585,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html</t>
@@ -561,6 +600,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>Kamal SAGUEM:</t>
         </r>
@@ -569,6 +609,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html</t>
@@ -583,6 +624,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html
 https://www.jumia.ma/samsung-galaxy-s26-ultra-69-16gb-ram-1-tb-rom-cobalt-violet-67758540.html
@@ -599,6 +641,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>Kamal SAGUEM:</t>
         </r>
@@ -607,6 +650,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t xml:space="preserve">
 https://www.jumia.ma/hisense-smart-tv-qled-4k-55-garantie-24-mois-67313922.html</t>
@@ -621,6 +665,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html
 https://www.jumia.ma/75-crystal-uhd-4k-smart-tv-one-ui-tizen-hdr10-design-metalstream-support-gratuit-75u8075-samsung-mpg1544568.html</t>
@@ -635,6 +680,7 @@
             <sz val="9"/>
             <color indexed="81"/>
             <rFont val="Tahoma"/>
+            <family val="2"/>
           </rPr>
           <t>https://www.jumia.ma/samsung-galaxy-tab-s9-ultra-12-go-512-go-graphite-65760372.html
 https://www.jumia.ma/samsung-galaxy-s26-ultra-69-16gb-ram-1-tb-rom-cobalt-violet-67758540.html
@@ -825,11 +871,13 @@
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
+      <family val="2"/>
     </font>
     <font>
       <sz val="9"/>
       <color indexed="81"/>
       <name val="Tahoma"/>
+      <family val="2"/>
     </font>
   </fonts>
   <fills count="5">
@@ -1236,6 +1284,28 @@
 </a:theme>
 </file>
 
+<file path=xl/webextensions/taskpanes.xml><?xml version="1.0" encoding="utf-8"?>
+<wetp:taskpanes xmlns:wetp="http://schemas.microsoft.com/office/webextensions/taskpanes/2010/11">
+  <wetp:taskpane dockstate="right" visibility="0" width="438" row="2">
+    <wetp:webextensionref xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+  </wetp:taskpane>
+</wetp:taskpanes>
+</file>
+
+<file path=xl/webextensions/webextension1.xml><?xml version="1.0" encoding="utf-8"?>
+<we:webextension xmlns:we="http://schemas.microsoft.com/office/webextensions/webextension/2010/11" id="{2E6A55FA-44E5-4144-B938-C5C2AFF1ECAF}">
+  <we:reference id="WA200009404" version="1.0.0.8" store="Omex" storeType="OMEX"/>
+  <we:alternateReferences>
+    <we:reference id="WA200009404" version="1.0.0.8" store="WA200009404" storeType="OMEX"/>
+  </we:alternateReferences>
+  <we:properties>
+    <we:property name="claude.fileId" value="&quot;a96eb725-f485-4d31-ac4e-1af434826f94&quot;"/>
+  </we:properties>
+  <we:bindings/>
+  <we:snapshot xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships"/>
+</we:webextension>
+</file>
+
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{3F6CAD69-D52B-4CD1-ADB7-85227535F7C6}">
   <dimension ref="A1:D15"/>

</xml_diff>